<commit_message>
- Initilized a sql3 DB for creating table and inseting AIS data. - Excellhas now his own manager seperated from sql3 DB.
</commit_message>
<xml_diff>
--- a/AIS_Response_Manager/AIS-Responder_Data - BackUp.xlsx
+++ b/AIS_Response_Manager/AIS-Responder_Data - BackUp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\borag\Downloads\Shool_2025-2026\Stage_2026\GIT\BoatRadar_Project\AIS_Response_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44F39627-BAF8-4D28-BAC3-273F1F1563BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511A509B-7E2B-4FF6-8491-BC9B1E473C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{511D1754-1C3F-4502-B4DA-96103ADE0086}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{511D1754-1C3F-4502-B4DA-96103ADE0086}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>ID</t>
   </si>
@@ -90,9 +90,6 @@
   </si>
   <si>
     <t>0s</t>
-  </si>
-  <si>
-    <t>null</t>
   </si>
   <si>
     <t>28.8 NMI</t>
@@ -552,31 +549,19 @@
         <v>16</v>
       </c>
       <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
         <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>22</v>
       </c>
       <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>18</v>
       </c>
-      <c r="J2" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>19</v>
-      </c>
-      <c r="M2" t="s">
-        <v>20</v>
-      </c>
-      <c r="N2" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>